<commit_message>
Record Operation Omegaline seizure of Virtualine (Oct 2026)
- Railnet/Virtualine row: status flagged -> seized; DOJ aliases, seized
  domain, Dutch server seizure, TRM/Chainalysis payment findings,
  AS202412 post-seizure routing, DROP-listed prefixes, current
  neighbours, and AS219199 recorded as an unconfirmed lead
- KPROHOST, metaspinner AS209800 and Pfcloud rows: seizure context
- SOURCE_INDEX: nine sources for the operation and the 2026-10-29
  routing/registry checks; statistics updated
- TIMELINE, ECOSYSTEM_MAP (3.2, 3.7, peering, appendices), README,
  taxonomy and playbook updated; anonrdp.com seizure noted as a lead
- BPH_Master.xlsx regenerated; validate_repo.py passes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xUWs6GeU36Hc3VWSoeuH2
</commit_message>
<xml_diff>
--- a/BPH_Master.xlsx
+++ b/BPH_Master.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BPH_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BPH_Master" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>flagged</t>
+          <t>seized</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1627,17 +1627,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AS202412 (OMEGATECH / Omegatech LTD [SC]; live Virtualine network, Spamhaus ASN-DROP under virtualine.org)</t>
+          <t>AS202412 (OMEGATECH / Omegatech LTD [SC]; Virtualine network until the Oct 2026 seizure - seen by 1 of 323 RIS peers since 2026-10-27; Spamhaus ASN-DROP under virtualine.org)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Originated by AS202412 Jan-Oct 2026, all on Spamhaus DROP (2026-10-29): 91.92.240.0/22; 158.94.208.0/22; 178.16.52.0/22 (these three ex-AS209800); 45.132.180.0/24; 94.26.38.0/24; 94.154.35.0/24; 94.154.40.0/24; 94.154.46.0/24; 130.12.180.0/24; 146.19.125.0/24; 193.30.241.0/24. Also short-lived /24s from broker-leased space that moves between unrelated ASNs (re-check the current origin before blocking): 45.74.7.0/24; 45.74.57.0/24; 45.74.59.0/24; 104.250.184.0/24; 172.111.246.0/24</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>United States (Kentucky LLC)</t>
+          <t>United States (Kentucky LLC: Railnet); Seychelles (Omegatech LTD, RIPE org created 2026-01-05)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Russia-linked operator; EU-hosted infrastructure</t>
+          <t>Russian-speaking operator; EU-hosted infrastructure (Dutch servers in Limburg seized Oct 2026)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1647,12 +1652,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Virtualine Technologies; RAILNET; OMEGATECH; DripHosting/DiorHost; RetryHost</t>
+          <t>Virtualine Technologies; RAILNET; OMEGATECH; Secury; Massgod; Spamhouse; Lanedo; DripHosting/DiorHost; RetryHost; virtualine.net (seized); virtualine.org</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>aurologic GmbH (AS30823) (~95% of prefixes, Aug 2025); Pfcloud UG (AS51396) (one /24)</t>
+          <t>Pfcloud UG (AS51396) and PEERYX NETWORK SAS (AS213382) (AS202412 neighbours, Oct 2026); aurologic GmbH (AS30823) (~95% of prefixes, Aug 2025; still a DDoS-protection tunnel hop in a community traceroute, Oct 2026)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1660,29 +1665,39 @@
           <t>aurologic GmbH</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>FBI seizure of virtualine.net under an E.D. Va. warrant (Operation Omegaline), announced Oct 27 2026; Politie Midden-Nederland seized dozens of physical servers in Limburg (hundreds of VPS offline; data on 3,000+ customers); concurrent FBI and German police actions against suspects and crypto - no operators named or charges announced</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>UAC-0050; UAC-0006</t>
+          <t>UAC-0050; UAC-0006; 'Vendor 1' CSAM/NCII and hack-for-hire forum (DOJ); Russian drug marketplace, sextortion scheme and ransomware groups (crypto payers, TRM)</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Latrodectus; AsyncRAT</t>
+          <t>Latrodectus; AsyncRAT; StealC (crypto payer, TRM)</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Underground forum advertising; Prefix shedding; No route diversification</t>
+          <t>Underground forum advertising; Prefix shedding; No route diversification; Shell-company migration sold as a service; No-AML bitcoin payments</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Spamhaus ASN-DROP (AS202412 under virtualine.org; AS214943 and AS214940 listed under virtualine.org in Dec 2025); Underground forum advertising; High malicious traffic ratio</t>
+          <t>Spamhaus ASN-DROP (AS202412 under virtualine.org; AS214943 and AS214940 listed under virtualine.org in Dec 2025); Every AS202412-originated prefix on Spamhaus DROP; Underground forum advertising; High malicious traffic ratio; LE seizure</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1692,12 +1707,17 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>RF-TAE-2026; GBHACKERS-BPH; TEAMCYMRU-VIRTUALINE; SPAMHAUS-BPH; RF-AUROLOGIC; SPAMHAUS-ASNDROP-2026; INTRINSEC-OMEGATECH-2026; INTRINSEC-UAC-2025; REGISTRY-SNAPSHOT-2026-09; INTRINSEC-FDN3-2025</t>
+          <t>RF-TAE-2026; GBHACKERS-BPH; TEAMCYMRU-VIRTUALINE; SPAMHAUS-BPH; RF-AUROLOGIC; SPAMHAUS-ASNDROP-2026; INTRINSEC-OMEGATECH-2026; INTRINSEC-UAC-2025; REGISTRY-SNAPSHOT-2026-09; INTRINSEC-FDN3-2025; DOJ-VIRTUALINE-2026; POLITIE-VIRTUALINE-2026; SILENTPUSH-OMEGATECH-2026; CHAINALYSIS-VIRTUALINE-2026; TRM-VIRTUALINE-2026; THERECORD-VIRTUALINE-2026; THN-VIRTUALINE-2026; LES-VIRTUALINE-2026; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Virtualine Technologies is the operator behind Railnet LLC (AS214943, Kentucky LLC), KPROHOST (AS214940), the 'metaspinner' AS209800 front, likely Karina Rashkovska (AS215789) and now OMEGATECH (AS202412) - at least five number-resource identities. Advertised on Russian-language forums for phishing/spam enablement ('DMCA &amp; Abuse Ignored'). RF ranked Virtualine #1 by Threat Density for 2025; Intrinsec documented UAC-0050/UAC-0006 activity on its infrastructure and, in May 2026, assessed OMEGATECH as 'yet another network created by Virtualine' (642k+ honeypot hits in March 2026). In April 2025 it shifted IPv4 resources to the 'metaspinner' AS209800; those ranges now sit on AS202412. AS214943 has announced nothing since ~2026-02 and was dropped from ASN-DROP; OMEGATECH is the live network (15 /24s, 13 on Spamhaus DROP). Tier raised T2 -&gt; T1 on 2026-09-25 (taxonomy T1: RF top-decile density; forum BPH advertising with infrastructure evidence; 3+ independent vendors). | Merged record (was a duplicate AS214943 row).</t>
+          <t>Virtualine Technologies is the operator behind Railnet LLC (AS214943, Kentucky LLC), KPROHOST (AS214940), the 'metaspinner' AS209800 front, likely Karina Rashkovska (AS215789) and OMEGATECH (AS202412) - at least five number-resource identities. SEIZED 2026-10-27 (Operation Omegaline): the FBI Washington Field Office seized virtualine.net under an E.D. Va. warrant, with Polizei Hessen, Politie Midden-Nederland, the UK NCA and private partners OverRIPE and Lumen; Chainalysis supported. DOJ names the aliases Secury, Massgod, Spamhouse, Lanedo and Omegatech, alleges it knowingly hosted 'Vendor 1' (a forum selling CSAM and non-consensual intimate images, with hack-for-hire) despite notices from German, Canadian and Australian police, NCMEC and a victim's attorney from Jan 2026, and that it laundered customer payments taken via unhosted 'BTC [NO-AML]' addresses. Forum advertising: Exploit.in from 2024-08-28 ('all illegal/black hat activities ... except for child contents and terrorism', Sept 2024); HackForums ('ignored more abuse than your last three therapists', June 2025); in Mar 2026 it sold an 'additional protection plan' moving a customer's server to an unaffiliated shell company after an LE request. Dutch police seized dozens of physical servers in Limburg (hundreds of VPS offline; data on 3,000+ customers) and say the FBI and German police acted against suspects and crypto at the same time; no operators were named or charged. TRM: most illicit-attributed crypto of any TRM-labelled BPH in 2026 (inflows ~44% Russian drug market, ~17% sextortion, ~13% mixer, ~5% ransomware; also StealC and the BPH Volhav). Network: Silent Push saw the move from AS214943 to AS202412 on 2026-02-11; AS202412 originated 24 /24s in the two weeks before the seizure (all on Spamhaus DROP) and has been seen by 1 of 323 RIS peers since 2026-10-27; its last neighbours were Pfcloud (AS51396) and PEERYX (AS213382). The operator posted an open letter on virtualine.org denying the allegations and saying it could rebrand in 'a day, perhaps even less' - watch for a successor ASN. LEAD (not attributed): AS219199 (GENYUS SOFT LTD [SC], created 2026-07-15) announced four broker-leased /24s from 2026-10-22, including 172.111.246.0/24 previously on AS202412, and withdrew them on the morning of the seizure; only a community post calls it Virtualine, and Spamhaus lists it under genyus.sc. Earlier history: RF ranked Virtualine #1 by Threat Density for 2025; Intrinsec documented UAC-0050/UAC-0006 activity and in May 2026 assessed OMEGATECH as 'yet another network created by Virtualine'; in April 2025 it shifted IPv4 resources to AS209800 (Spamhaus reported the expansion in Sept 2025), and those ranges later moved to AS202412. Status flagged -&gt; seized 2026-10-29; tier stays T1 (raised T2 -&gt; T1 on 2026-09-25). | Merged record (was a duplicate AS214943 row).</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Russian-speaking bulletproof host (RF 2025 Threat Density #1); domain seized and Dutch servers taken in the FBI-led Operation Omegaline, Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -2102,17 +2122,17 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>RF-TAE-2026; RF-AUROLOGIC; KREBS-BPH; REGISTRY-SNAPSHOT-2026-09</t>
+          <t>RF-TAE-2026; RF-AUROLOGIC; KREBS-BPH; REGISTRY-SNAPSHOT-2026-09; DOJ-VIRTUALINE-2026; THN-VIRTUALINE-2026</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>AS209800 was created 2025-04-25 and announced solely via aurologic; RF Insikt says it was controlled by Virtualine-affiliated actors who impersonated the long-standing legitimate Hamburg company metaspinner net GmbH (RENAMED 2026-09-25 so the row no longer names that company as the operator). Its prefixes (91.92.240.0/22, 158.94.208.0/22, 178.16.52.0/22) received Virtualine traffic from April 2025 and now originate from OMEGATECH AS202412 (see the Railnet/Virtualine row). The ASN has been re-issued to an unrelated German GbR (ZEMA) - do not block AS209800. Status set to 'dissolved' (network defunct).</t>
+          <t>AS209800 was created 2025-04-25 and announced solely via aurologic; RF Insikt says it was controlled by Virtualine-affiliated actors who impersonated the long-standing legitimate Hamburg company metaspinner net GmbH (RENAMED 2026-09-25 so the row no longer names that company as the operator). Its prefixes (91.92.240.0/22, 158.94.208.0/22, 178.16.52.0/22) received Virtualine traffic from April 2025 and now originate from OMEGATECH AS202412 (see the Railnet/Virtualine row). The ASN has been re-issued to an unrelated German GbR (ZEMA) - do not block AS209800. Status set to 'dissolved' (network defunct). Attribution strengthened 2026-10-29: DOJ lists 'Lanedo' among Virtualine's aliases, matching the LANEDONET re-description, and Spamhaus (Sept 2025) reported Virtualine's expansion onto AS209800. Tier left at T3 as a historical record pending review.</t>
         </is>
       </c>
     </row>
@@ -2179,17 +2199,17 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>RF-AUROLOGIC; RIPE-DB; SPAMHAUS-ASNDROP-2026; REGISTRY-SNAPSHOT-2026-09; INTRINSEC-FDN3-2025</t>
+          <t>RF-AUROLOGIC; RIPE-DB; SPAMHAUS-ASNDROP-2026; REGISTRY-SNAPSHOT-2026-09; INTRINSEC-FDN3-2025; DOJ-VIRTUALINE-2026</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>RIPE-registered 2024-05-10 by KPROHOST LLC (Frankfort, KY; Kentucky reg. 1360766); abuse contact kprohost.abuse@gmail.com. Intrinsec attributes AS214940 to Virtualine, and Spamhaus listed it under virtualine.org in Dec 2025 (since delisted). Its two historical /24s (195.211.191.0/24, 45.144.212.0/24) now originate from HBING (AS208949) and Pfcloud (AS51396). The ASN has announced nothing since ~2026-08-12. Tier raised T3 -&gt; T2 on 2026-09-25 (shell structure; part of a T1 operator; blocklisting). Correction: its upstreams were Pfcloud and AS215436, not aurologic.</t>
+          <t>RIPE-registered 2024-05-10 by KPROHOST LLC (Frankfort, KY; Kentucky reg. 1360766); abuse contact kprohost.abuse@gmail.com. Intrinsec attributes AS214940 to Virtualine, and Spamhaus listed it under virtualine.org in Dec 2025 (since delisted). Its two historical /24s (195.211.191.0/24, 45.144.212.0/24) now originate from HBING (AS208949) and Pfcloud (AS51396). The ASN has announced nothing since ~2026-08-12. Tier raised T3 -&gt; T2 on 2026-09-25 (shell structure; part of a T1 operator; blocklisting). Correction: its upstreams were Pfcloud and AS215436, not aurologic. Virtualine, the operator, was disrupted in the FBI-led Operation Omegaline on 2026-10-27 (see the Railnet/Virtualine row); AS214940 was already dark.</t>
         </is>
       </c>
     </row>
@@ -5063,17 +5083,17 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>RUDIS-BPH-WATCH; RF-AUROLOGIC; SPAMHAUS-ASNDROP-2026; GREYNOISE-WEEKLY-2026-08; GREYNOISE-REACT2SHELL-2026; REGISTRY-SNAPSHOT-2026-09</t>
+          <t>RUDIS-BPH-WATCH; RF-AUROLOGIC; SPAMHAUS-ASNDROP-2026; GREYNOISE-WEEKLY-2026-08; GREYNOISE-REACT2SHELL-2026; REGISTRY-SNAPSHOT-2026-09; REGISTRY-SNAPSHOT-2026-10; LES-VIRTUALINE-2026</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>German micro-provider (AS51396: 26 IPv4 and 24 IPv6 prefixes). Spamhaus ASN-DROP has listed AS51396 since at least Feb 2024 (with a since-recycled AS202685 'as-pfcloud'); it now also lists AS215310 (USERCLOUD) and AS400328 (Intelligence Hosting LLC) under pfcloud.io. RF lists Pfcloud as an upstream of the Virtualine/Railnet 'hosting island' alongside aurologic. GreyNoise (Aug 2026): 204.76.203.43 on AS51396 generated 393,777 sessions and most of the period's 121,068 Hikvision CVE-2021-36260 exploitation attempts; Pfcloud IPs also appear among React2Shell sources. A community note (Sept 2026, D-grade) describes a Pfcloud open directory staging FortiGate 60F exploit modules on an IP previously listed as AsyncRAT C2. Tier raised T3 -&gt; T2 (status flagged) on 2026-09-25 per the ASN-DROP escalation rule; the earlier single-honeypot caveat is outdated.</t>
+          <t>German micro-provider (AS51396: 26 IPv4 and 24 IPv6 prefixes). Spamhaus ASN-DROP has listed AS51396 since at least Feb 2024 (with a since-recycled AS202685 'as-pfcloud'); it now also lists AS215310 (USERCLOUD) and AS400328 (Intelligence Hosting LLC) under pfcloud.io. RF lists Pfcloud as an upstream of the Virtualine/Railnet 'hosting island' alongside aurologic. GreyNoise (Aug 2026): 204.76.203.43 on AS51396 generated 393,777 sessions and most of the period's 121,068 Hikvision CVE-2021-36260 exploitation attempts; Pfcloud IPs also appear among React2Shell sources. A community note (Sept 2026, D-grade) describes a Pfcloud open directory staging FortiGate 60F exploit modules on an IP previously listed as AsyncRAT C2. Tier raised T3 -&gt; T2 (status flagged) on 2026-09-25 per the ASN-DROP escalation rule; the earlier single-honeypot caveat is outdated. Oct 2026: Pfcloud was one of the last two neighbours of Virtualine's AS202412 when it was seized (Operation Omegaline); a community post says the Dutch servers seized in Limburg were Tube-Hosting (AS49581) hardware resold to Virtualine through Pfcloud (unconfirmed).</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">

</xml_diff>

<commit_message>
Raise metaspinner-named AS209800 front from T3 to T2
Matches the other Virtualine sub-networks (KPROHOST, Karina
Rashkovska): an operator-controlled front with an impersonated
identity, no route diversification and all three former /22s on
Spamhaus DROP, on RF (B) and Spamhaus (C) evidence plus the DOJ
"Lanedo" alias. Status stays dissolved; the ASN stays marked
historical/reassigned. Taxonomy T2/T3 counts, ecosystem map
appendices and BPH_Master.xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xUWs6GeU36Hc3VWSoeuH2
</commit_message>
<xml_diff>
--- a/BPH_Master.xlsx
+++ b/BPH_Master.xlsx
@@ -2067,7 +2067,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>T3-Suspected</t>
+          <t>T2-High Risk</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Impersonated corporate identity; No route diversification; ASN since reassigned</t>
+          <t>Impersonated corporate identity; No route diversification; ASN since reassigned; Former prefixes on Spamhaus DROP</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2122,17 +2122,17 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>RF-TAE-2026; RF-AUROLOGIC; KREBS-BPH; REGISTRY-SNAPSHOT-2026-09; DOJ-VIRTUALINE-2026; THN-VIRTUALINE-2026</t>
+          <t>RF-TAE-2026; RF-AUROLOGIC; KREBS-BPH; REGISTRY-SNAPSHOT-2026-09; DOJ-VIRTUALINE-2026; THN-VIRTUALINE-2026; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>AS209800 was created 2025-04-25 and announced solely via aurologic; RF Insikt says it was controlled by Virtualine-affiliated actors who impersonated the long-standing legitimate Hamburg company metaspinner net GmbH (RENAMED 2026-09-25 so the row no longer names that company as the operator). Its prefixes (91.92.240.0/22, 158.94.208.0/22, 178.16.52.0/22) received Virtualine traffic from April 2025 and now originate from OMEGATECH AS202412 (see the Railnet/Virtualine row). The ASN has been re-issued to an unrelated German GbR (ZEMA) - do not block AS209800. Status set to 'dissolved' (network defunct). Attribution strengthened 2026-10-29: DOJ lists 'Lanedo' among Virtualine's aliases, matching the LANEDONET re-description, and Spamhaus (Sept 2025) reported Virtualine's expansion onto AS209800. Tier left at T3 as a historical record pending review.</t>
+          <t>AS209800 was created 2025-04-25 and announced solely via aurologic; RF Insikt says it was controlled by Virtualine-affiliated actors who impersonated the long-standing legitimate Hamburg company metaspinner net GmbH (RENAMED 2026-09-25 so the row no longer names that company as the operator). Its prefixes (91.92.240.0/22, 158.94.208.0/22, 178.16.52.0/22) received Virtualine traffic from April 2025 and now originate from OMEGATECH AS202412 (see the Railnet/Virtualine row). The ASN has been re-issued to an unrelated German GbR (ZEMA) - do not block AS209800. Status set to 'dissolved' (network defunct). Attribution strengthened 2026-10-29: DOJ lists 'Lanedo' among Virtualine's aliases, matching the LANEDONET re-description, and Spamhaus (Sept 2025) reported Virtualine's expansion onto AS209800. Tier raised T3 -&gt; T2 on 2026-10-30 to match the other Virtualine sub-networks (KPROHOST, Karina Rashkovska): an operator-controlled front with obscured ownership (impersonated identity), no route diversification and all three former /22s on Spamhaus DROP, on RF (B) and Spamhaus (C) evidence plus the DOJ alias. Kept as a historical record - status stays 'dissolved'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify previously unconfirmed items; correct EU 21st platform count
- Dabai: RF's founding estimate (Dec 2024) and 19,225-member figure
  confirmed in the report; caveat removed
- Tudou: Elliptic states Huione Guarantee acquired a 30% stake in
  Dec 2024; caveat removed in notes and parent_entity
- A7A5: EU 21st package A7 designations (incl. A7 Nigeria and A7
  Africa, per TRM) added; Yandex data-centre strikes and the reported
  collapse in A7A5 exchange activity recorded as C-grade
- EU 21st package: transaction ban covers 14 crypto platforms, not 11
  (Council/EEAS text) - corrected in TIMELINE and SOURCE_INDEX
- 3 new sources; TIMELINE entry for the A7A5 disruption

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xUWs6GeU36Hc3VWSoeuH2
</commit_message>
<xml_diff>
--- a/BPH_Master.xlsx
+++ b/BPH_Master.xlsx
@@ -4601,7 +4601,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>UK May 2025 (A7) and Aug 20 2025 (Old Vector LLC); EU July 2025 (A7) and 19th package Oct 23 2025 (full A7A5 transaction ban from Nov 25 2025); OFAC Aug 14 2025 (Old Vector LLC, A7 LLC, A71 LLC, A7 Agent LLC); OFAC Oct 1 2026: whole A7 Network designated a significant transnational criminal organization (E.O. 13581; Operation Economic Outcast); FinCEN Oct 1 2026: section 9714(a) proposed rule against A7 Network Sub-Agents plus an Alert</t>
+          <t>UK May 2025 (A7) and Aug 20 2025 (Old Vector LLC); EU July 2025 (A7) and 19th package Oct 23 2025 (full A7A5 transaction ban from Nov 25 2025); EU 21st package Jul 23 2026 (four A7-network designations incl. A7 Nigeria and A7 Africa; transaction ban on 14 crypto platforms); OFAC Aug 14 2025 (Old Vector LLC, A7 LLC, A71 LLC, A7 Agent LLC); OFAC Oct 1 2026: whole A7 Network designated a significant transnational criminal organization (E.O. 13581; Operation Economic Outcast); FinCEN Oct 1 2026: section 9714(a) proposed rule against A7 Network Sub-Agents plus an Alert</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4626,12 +4626,12 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>OFAC-GARANTEX; CHAINALYSIS-A7A5; TRM-A7A5-2026; OFAC-A7-NETWORK-2026</t>
+          <t>OFAC-GARANTEX; CHAINALYSIS-A7A5; TRM-A7A5-2026; OFAC-A7-NETWORK-2026; EU-21ST-PACKAGE; TRM-EU21-2026; CRYPTOPOLITAN-A7A5-2026; ALJAZEERA-YANDEX-2026</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>Russian ruble-backed stablecoin issued by Kyrgyzstan's Old Vector; A7 LLC is the token's creator. Chainalysis (2026 Crypto Crime Report): $93.3B moved 'in less than a year'; Elliptic: more than $100B in under a year (the $93.1B and $72B figures elsewhere are earlier snapshots). Garantex moved funds into A7A5 from as early as January 2025 (TRM). The no-KYC Instant Swapper reportedly converted &gt;$2.2B of A7A5 into mainstream USD stablecoins (unverified). The EU banned A7A5 transactions from 2025-11-25. Its economy ran through Grinex, and on-chain volume reportedly collapsed after Grinex suspended in April 2026 (the '~96%' decline figure is attributed to Elliptic in secondary reporting). On 2026-10-01 Treasury designated the whole A7 Network as a transnational criminal organization: its Sub-Agents processed more than $17B (Jan 2025-Jun 2026) and 'catered to cybercriminals, including ransomware' actors, and the network is linked to Nobitex and to North Korean hacks; FinCEN proposed cutting Sub-Agents off from US transmittals (rule not yet final). A7 LLC, A71 LLC and A7 Agent LLC are separately designated related entities, not aliases.</t>
+          <t>Russian ruble-backed stablecoin issued by Kyrgyzstan's Old Vector; A7 LLC is the token's creator. Chainalysis (2026 Crypto Crime Report): $93.3B moved 'in less than a year'; Elliptic: more than $100B in under a year (the $93.1B and $72B figures elsewhere are earlier snapshots). Garantex moved funds into A7A5 from as early as January 2025 (TRM). The no-KYC Instant Swapper reportedly converted &gt;$2.2B of A7A5 into mainstream USD stablecoins (unverified). The EU banned A7A5 transactions from 2025-11-25. Its economy ran through Grinex, and on-chain volume reportedly collapsed after Grinex suspended in April 2026 (the '~96%' decline figure is attributed to Elliptic in secondary reporting). On 2026-10-01 Treasury designated the whole A7 Network as a transnational criminal organization: its Sub-Agents processed more than $17B (Jan 2025-Jun 2026) and 'catered to cybercriminals, including ransomware' actors, and the network is linked to Nobitex and to North Korean hacks; FinCEN proposed cutting Sub-Agents off from US transmittals (rule not yet final). Ukrainian drone strikes on Yandex data centres (Sasovo, 2026-10-08, and Kaluga the same week) disrupted A7A5's exchange service, which Elliptic's Tom Robinson says is hosted there: crypto press citing Robinson and Etherscan/Tronscan data report daily transfers falling from about 600 to about 61, mostly DEX swaps, and holders unpaid interest since 2026-10-09 (Elliptic's own write-up not read; figures C-grade). A7 LLC, A71 LLC and A7 Agent LLC are separately designated related entities, not aliases.</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W57" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>Recorded Future/Insikt: major Chinese-language guarantee (danbao) Telegram marketplace resembling the defunct Huione Guarantee, with thousands of thematic channels (overseas phishing, laundering, 'sweeping' goods in Japan and South Korea) and a search bot. The RF report appears to date from about April 2026 (the relaying digest is dated 2026-04-23), not February. Reported emergence ~Dec 2024 and ~19,225 members in its largest group are unverified. Flare counts more than 30 marketplaces that emerged after Huione Guarantee ceased operations in May 2025; Xinbi (disrupted by the US on 2026-09-09) is the largest of the successors.</t>
+          <t>Recorded Future/Insikt: major Chinese-language guarantee (danbao) Telegram marketplace resembling the defunct Huione Guarantee, with thousands of thematic channels (overseas phishing, laundering, 'sweeping' goods in Japan and South Korea) and a search bot. The RF report appears to date from about April 2026 (the relaying digest is dated 2026-04-23), not February. RF says Dabai was likely founded in December 2024 (based on its Telegram channel's creation date) and counted 19,225 members in its 'Dabai Guarantee Big Group' (@dabai_c) at the time of writing (verified 2026-10-30). Flare counts more than 30 marketplaces that emerged after Huione Guarantee ceased operations in May 2025; Xinbi (disrupted by the US on 2026-09-09) is the largest of the successors.</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Huione / Haowang Guarantee (announced a stake in Dec 2024; 30% figure unverified)</t>
+          <t>Huione / Haowang Guarantee (announced a stake in Dec 2024; 30% stake per Elliptic)</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W58" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>Huione's designated successor: in December 2024 Haowang (ex-Huione) Guarantee announced it was buying a stake in Tudou (FinCEN; the 30% figure is unverified). Processed &gt;$12B - the third-largest illicit marketplace ever (Elliptic). In January 2026, after Prince Group chairman Chen Zhi was arrested in Cambodia and extradited to China (reported 2026-01-07), Tudou effectively ceased transactions through its public Telegram groups and admin-wallet activity collapsed; gambling operations continue and Elliptic says it remains to be seen whether this is a full shutdown or a pivot. Status corrected dissolved -&gt; flagged on 2026-09-25 (no legal dissolution documented).</t>
+          <t>Huione's designated successor: in December 2024 Haowang (ex-Huione) Guarantee announced it was buying a stake in Tudou (FinCEN; Elliptic gives the size as a 30% stake, acquired by Huione Guarantee in December 2024 - verified 2026-10-30). Processed &gt;$12B - the third-largest illicit marketplace ever (Elliptic). In January 2026, after Prince Group chairman Chen Zhi was arrested in Cambodia and extradited to China (reported 2026-01-07), Tudou effectively ceased transactions through its public Telegram groups and admin-wallet activity collapsed; gambling operations continue and Elliptic says it remains to be seen whether this is a full shutdown or a pivot. Status corrected dissolved -&gt; flagged on 2026-09-25 (no legal dissolution documented).</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">

</xml_diff>

<commit_message>
Resolve registry-checkable caveats (audit part 2, in progress)
- Datavice: AS206336 confirmed as registered to DATAVICE MCHJ since
  2025-07-18 (Datavice LIR; org references aeza-mnt); added as its ASN
- Phanes: AS64425 handed 45.148.120.0/24 and 45.148.123.0/24 to
  AS49042 in April 2023 (routing history)
- SHANGXING: APNIC record confirmed; unsupported PEG TECH and
  'AS Data HK' links removed
- SWISSNETWORK02: no registry or geolocation evidence for Switzerland
- Cloudzy: Wyoming registration per CyberScoop
- AnonRDP: Blatant-announced 46.151.182.0/24 is registered to Ghosty
  Networks LLC (GHOSTYNETWORKS-MNT); Host Baltic claim still
  unconfirmed (no Lithuanian geolocation)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xUWs6GeU36Hc3VWSoeuH2
</commit_message>
<xml_diff>
--- a/BPH_Master.xlsx
+++ b/BPH_Master.xlsx
@@ -2000,7 +2000,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>United States (incorporated; Wyoming unverified)</t>
+          <t>United States (Wyoming; registered under a registered-agent lawyer per CyberScoop/Halcyon)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2964,17 +2964,17 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>OSINT-REVIEWS; REGISTRY-SNAPSHOT-2026-09</t>
+          <t>OSINT-REVIEWS; REGISTRY-SNAPSHOT-2026-09; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Dutch hoster (reported address Keteldiep 15, Urk) rebranded from Flaunt7. AS49042 was historically 'Phanes Networks B.V.' and is now absent from the registry and routing data. Silent Push reports 'bulletproof' in Phanes' marketing and a 4-day abuse response; Trustpilot reviews document unresponsive handling of phishing complaints. SpectraIP is its peering partner, not an alias. SKB Enterprise B.V. held a separate ASN (AS64425) and its relationship to Phanes is unverified.</t>
+          <t>Dutch hoster (reported address Keteldiep 15, Urk) rebranded from Flaunt7. AS49042 was historically 'Phanes Networks B.V.' and is now absent from the registry and routing data. Silent Push reports 'bulletproof' in Phanes' marketing and a 4-day abuse response; Trustpilot reviews document unresponsive handling of phishing complaints. SpectraIP is its peering partner, not an alias. SKB Enterprise B.V. held a separate ASN (AS64425, now unregistered): routing history shows AS64425 announcing 45.148.120.0/24 and 45.148.123.0/24 until 2023-04-28 and Phanes' AS49042 announcing the same prefixes from 2023-04-17, with both ASNs going silent in Sept 2025 - the two carried the same address space (RIPEstat, checked 2026-10-30).</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Switzerland (claimed; unverified); aurologic-transited</t>
+          <t>Switzerland claimed only by the SWISSNETWORK name - no registry or geolocation evidence (its former /22s geolocated to DE, GB, FR, KZ, US, RU, UZ and UA, and have since been returned); aurologic-transited</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5441,6 +5441,11 @@
           <t>T1-Confirmed BPH</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>AS206336 (Datavice; registered to DATAVICE MCHJ [UZ] since 2025-07-18; no routes)</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr">
         <is>
           <t>Uzbekistan</t>
@@ -5493,17 +5498,17 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>OFAC-MEDIALAND</t>
+          <t>OFAC-MEDIALAND; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>Uzbekistan-registered (Tashkent) Aeza expansion entity. OFAC SDN record: established 2025-07-03; Tax ID 312252645; Business Registration 2868352; address 3 Irrigator Massive, Hamid Olimjon MFY, Tashkent; programs CYBER4 and CAATSA-RUSSIA; 'Linked To: AEZA GROUP LLC'. Designated 2025-11-19 alongside Hypercore Ltd, Smart Digital Ideas DOO, Maksim Makarov and Ilya Zakirov; absent from the UK's 19 Nov 2025 notices (OFAC-only). No ASN is stated in the designation; the registry lists a dark AS206336 as 'DATAVICE MCHJ', but per-ASN metadata still shows a previous holder, so treat it as an unverified lead.</t>
+          <t>Uzbekistan-registered (Tashkent) Aeza expansion entity. OFAC SDN record: established 2025-07-03; Tax ID 312252645; Business Registration 2868352; address 3 Irrigator Massive, Hamid Olimjon MFY, Tashkent; programs CYBER4 and CAATSA-RUSSIA; 'Linked To: AEZA GROUP LLC'. Designated 2025-11-19 alongside Hypercore Ltd, Smart Digital Ideas DOO, Maksim Makarov and Ilya Zakirov; absent from the UK's 19 Nov 2025 notices (OFAC-only). No ASN is stated in the designation, but the RIPE database assigns AS206336 to DATAVICE MCHJ (ORG-DM279-RIPE, Tashkent; aut-num re-created 2025-07-18, fifteen days after the company was established). Datavice is its own LIR (lir-uz-datavice-1-MNT), and its org object lists aeza-mnt among its referenced maintainers - a direct registry tie to Aeza. AS206336 has announced nothing since the re-registration (its 2017-2023 routing history belongs to a previous holder) and is not on Spamhaus ASN-DROP (checked 2026-10-30).</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -5759,17 +5764,17 @@
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>CV-GSHELL-2026-07; CV-OPENDIR-2026-09; GREYNOISE-REACT2SHELL-2026; C2INTELFEEDS; REGISTRY-SNAPSHOT-2026-09</t>
+          <t>CV-GSHELL-2026-07; CV-OPENDIR-2026-09; GREYNOISE-REACT2SHELL-2026; C2INTELFEEDS; REGISTRY-SNAPSHOT-2026-09; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>AS400619 is registered to AROSSCLOUD INC. (US) and originates 70 IPv4 prefixes (191,744 addresses), including 103.112.96.0/22 which covers the tracked 103.112.97.0/24; SHANGXING TECH LIMITED itself holds AS136452 and AS151468 (HK; neither announced), so the row name most likely reflects the inetnum holder while AROSSCLOUD owns the origin ASN (APNIC inetnum not yet confirmed). AS400619 and Fastmos (AS138644) tile 191.124.0.0/16 exactly between them - strong registry evidence of a shared reseller relationship. Hosts the July 2026 unreported Gshell C2 cluster (103.112.97.163/.199) and a Sept 2026 mass web-exploitation workspace (Fastmos :8889 - gen_targets/CVE-PoC/Java-memshell RCE-verify/k8s scan, 283KB target list) plus a second exploit box (AROSSCLOUD :9999) - first-party CrimsonVector open-directory hunts. Public corroboration: GreyNoise lists AS400619 among React2Shell exploitation sources (Jan 2026); C2IntelFeeds recorded Cobalt Strike C2s on AROSSCLOUD addresses (Aug-Sep 2026); community RAT feeds list several 103.112.97.x hosts. PEG TECH INC and 'AS Data HK' links are unverified.</t>
+          <t>AS400619 is registered to AROSSCLOUD INC. (US) and originates 70 IPv4 prefixes (191,744 addresses), including 103.112.96.0/22 which covers the tracked 103.112.97.0/24; SHANGXING TECH LIMITED itself holds AS136452 and AS151468 (HK; neither announced), so the row name most likely reflects the inetnum holder while AROSSCLOUD owns the origin ASN (confirmed: APNIC's record for 103.112.97.0/24, registered 2025-12-16, carries the name AROSS-AS with SHANGXING TECH LIMITED, Kwai Chung, Hong Kong, as administrative and technical contact). AS400619 and Fastmos (AS138644) tile 191.124.0.0/16 exactly between them - strong registry evidence of a shared reseller relationship. Hosts the July 2026 unreported Gshell C2 cluster (103.112.97.163/.199) and a Sept 2026 mass web-exploitation workspace (Fastmos :8889 - gen_targets/CVE-PoC/Java-memshell RCE-verify/k8s scan, 283KB target list) plus a second exploit box (AROSSCLOUD :9999) - first-party CrimsonVector open-directory hunts. Public corroboration: GreyNoise lists AS400619 among React2Shell exploitation sources (Jan 2026); C2IntelFeeds recorded Cobalt Strike C2s on AROSSCLOUD addresses (Aug-Sep 2026); community RAT feeds list several 103.112.97.x hosts. The earlier PEG TECH INC and 'AS Data HK' links were removed on 2026-10-30: neither appears among AS400619's neighbours or in the routing history of 103.112.96.0/22.</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr">
@@ -6040,17 +6045,17 @@
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>INTRINSEC-BTHOSTER; SPAMHAUS-ASNDROP-2026; REGISTRY-SNAPSHOT-2026-09; LES-VIRTUALINE-2026</t>
+          <t>INTRINSEC-BTHOSTER; SPAMHAUS-ASNDROP-2026; REGISTRY-SNAPSHOT-2026-09; LES-VIRTUALINE-2026; REGISTRY-SNAPSHOT-2026-10</t>
         </is>
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>Lithuanian hoster named by Intrinsec (June 2025) as a transit provider of the BtHoster/BTCloud AS-leasing operation (see the BtHoster row). Spamhaus ASN-DROP lists AS209605 (serveroffer.lt; 6 announced prefixes including 141.98.8.0/22 and 185.36.81.0/24, 5 of them overlapping Spamhaus DROP) and a newly listed Hong Kong sibling, AS135388 'RPL-HK' (RMP Protection Limited; 93.152.223.0/24 and 94.26.0.0/24). A second Host Baltic registration, AS211872 'ALPHA-NETWORKS', has no routes. Added 2026-09-25 as an upstream enabler (ASN-DROP inclusion plus upstream of a T1 entity, two independent sources). Oct 2026: a community post says AnonRDP's Lithuanian 'bulletproof' servers (see the AnonRDP / Blatant Technologies row) are hosted here and tunnelled through SMARTNET Germany - unconfirmed.</t>
+          <t>Lithuanian hoster named by Intrinsec (June 2025) as a transit provider of the BtHoster/BTCloud AS-leasing operation (see the BtHoster row). Spamhaus ASN-DROP lists AS209605 (serveroffer.lt; 6 announced prefixes including 141.98.8.0/22 and 185.36.81.0/24, 5 of them overlapping Spamhaus DROP) and a newly listed Hong Kong sibling, AS135388 'RPL-HK' (RMP Protection Limited; 93.152.223.0/24 and 94.26.0.0/24). A second Host Baltic registration, AS211872 'ALPHA-NETWORKS', has no routes. Added 2026-09-25 as an upstream enabler (ASN-DROP inclusion plus upstream of a T1 entity, two independent sources). Oct 2026: a community post says AnonRDP's Lithuanian 'bulletproof' servers (see the AnonRDP / Blatant Technologies row) are hosted here and tunnelled through SMARTNET Germany - unconfirmed (none of AS403005's prefixes geolocate to Lithuania; checked 2026-10-30).</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
@@ -6480,7 +6485,7 @@
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="W72" t="inlineStr">
@@ -6490,7 +6495,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>Self-styled 'bulletproof anonymous hosting' provider selling crypto-paid VPS/RDP, dedicated and web hosting, 'scanning' servers and a FastFlux CDN advertised as 'Spamhaus Ignored' (anonrdp.com registered 2023-10-04). Network lineage: Intrinsec (May 2026) found March 2026 malspam - a JavaScript backdoor aimed at CIS energy and finance ministries - sent from and controlled via the bulletproof US network GHOSTYNETWORKS (AS205759, Kentucky, registered Jan 2026), which it linked to the OPTIBOUNCE network previously tied to AnonRDP; Silent Push (Oct 2026) calls GHOSTYNETWORKS a shell company of AnonRDP and found the same four SPF addresses on anonrdp.com (Feb-Apr 2026) and ghostynetworks.com. AS205759 has since been deregistered. Current network: CrimsonVector DNS checks (2026-10-29) show solusvm.anonrdp.st and xmpp.anonrdp.st resolving into AS403005 (Blatant Technologies, LLC; ARIN-registered 2026-09-25, Seychelles registrant, Louisville KY contacts), and smtp/smtp01.anonrdp.st resolving to two of the ghostynetworks.com SPF addresses. AS403005 announces nine /24s, all on Spamhaus DROP, through a single upstream, SMARTNET Germany (AS203446); Spamhaus lists the ASN under blatant.host. A community post says the Lithuanian servers sit with UAB Host Baltic (AS209605, tracked here) - unconfirmed. Enforcement: on 2026-10-27, the day of the Virtualine seizure, the registry record for anonrdp.com was pointed at FBI seizure nameservers (13:13 UTC); no seizure page or DOJ statement had appeared by 2026-10-29. That day AnonRDP offered Virtualine customers a 'refugee offer' (it had also run a 'crazyrdp' promo code on 2025-11-15, days after the CrazyRDP seizure); on 2026-10-28 it moved to anonrdp.st, said a 'trusted source' warned it could be next, and said it had triggered an 'emergency kill switch' and was moving datacentres. Backup domains: anonrdp.net and an .onion address. Tier T1 (added 2026-10-29): LE domain seizure plus self-advertised bulletproof hosting with corroborating infrastructure, on Silent Push and Intrinsec (B) and registry/Spamhaus data (C). Status 'seized' covers the domain only - the operation is still running from anonrdp.st, so expect further ASN and prefix moves.</t>
+          <t>Self-styled 'bulletproof anonymous hosting' provider selling crypto-paid VPS/RDP, dedicated and web hosting, 'scanning' servers and a FastFlux CDN advertised as 'Spamhaus Ignored' (anonrdp.com registered 2023-10-04). Network lineage: Intrinsec (May 2026) found March 2026 malspam - a JavaScript backdoor aimed at CIS energy and finance ministries - sent from and controlled via the bulletproof US network GHOSTYNETWORKS (AS205759, Kentucky, registered Jan 2026), which it linked to the OPTIBOUNCE network previously tied to AnonRDP; Silent Push (Oct 2026) calls GHOSTYNETWORKS a shell company of AnonRDP and found the same four SPF addresses on anonrdp.com (Feb-Apr 2026) and ghostynetworks.com. AS205759 has since been deregistered. Current network: CrimsonVector DNS checks (2026-10-29) show solusvm.anonrdp.st and xmpp.anonrdp.st resolving into AS403005 (Blatant Technologies, LLC; ARIN-registered 2026-09-25, Seychelles registrant, Louisville KY contacts), and smtp/smtp01.anonrdp.st resolving to two of the ghostynetworks.com SPF addresses. AS403005 announces nine /24s, all on Spamhaus DROP, through a single upstream, SMARTNET Germany (AS203446); Spamhaus lists the ASN under blatant.host. The RIPE record for one of AS403005's /24s, 46.151.182.0/24 (netname Ghosty-24, created 2026-09-13), is maintained by GHOSTYNETWORKS-MNT for Ghosty Networks LLC (Scottsville, Kentucky) - a direct registry link between Blatant's network and GHOSTYNETWORKS; 31.56.19.0/24 is registered as BLATANT-NET to a Seychelles org. A community post says the Lithuanian servers sit with UAB Host Baltic (AS209605, tracked here); none of AS403005's prefixes geolocate to Lithuania, so this stays unconfirmed. Enforcement: on 2026-10-27, the day of the Virtualine seizure, the registry record for anonrdp.com was pointed at FBI seizure nameservers (13:13 UTC); no seizure page or DOJ statement had appeared by 2026-10-29. That day AnonRDP offered Virtualine customers a 'refugee offer' (it had also run a 'crazyrdp' promo code on 2025-11-15, days after the CrazyRDP seizure); on 2026-10-28 it moved to anonrdp.st, said a 'trusted source' warned it could be next, and said it had triggered an 'emergency kill switch' and was moving datacentres. Backup domains: anonrdp.net and an .onion address. Tier T1 (added 2026-10-29): LE domain seizure plus self-advertised bulletproof hosting with corroborating infrastructure, on Silent Push and Intrinsec (B) and registry/Spamhaus data (C). Status 'seized' covers the domain only - the operation is still running from anonrdp.st, so expect further ASN and prefix moves.</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">

</xml_diff>